<commit_message>
ajout du 3eme persona dans le storymap perturbation j-1
</commit_message>
<xml_diff>
--- a/IPSSI_APOCAL_KIT/docs/cadrage/04-story-map.xlsx
+++ b/IPSSI_APOCAL_KIT/docs/cadrage/04-story-map.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
   <si>
     <t>STORY MAP – EduTutor IA</t>
   </si>
@@ -291,6 +291,63 @@
   <si>
     <t>US-E11
 Prédire automatiquement la réussite à l'examen.</t>
+  </si>
+  <si>
+    <t>1. Valider la conformité</t>
+  </si>
+  <si>
+    <t>3. Piloter l'établissement</t>
+  </si>
+  <si>
+    <t>2. Gérer l'adoption</t>
+  </si>
+  <si>
+    <t>US-D01
+Vérifier que la solution est conforme au RGPD.</t>
+  </si>
+  <si>
+    <t>US-D02
+Déployer la solution auprès des enseignants.</t>
+  </si>
+  <si>
+    <t>US-D03
+Consulter les statistiques globales d'utilisation de l'établissement.</t>
+  </si>
+  <si>
+    <t>US-D04
+Consulter les engagements de sécurité et les CGU.</t>
+  </si>
+  <si>
+    <t>US-D05
+Suivre le taux d'adoption par les enseignants.</t>
+  </si>
+  <si>
+    <t>US-D06
+Exporter un rapport pour le conseil d'administration.</t>
+  </si>
+  <si>
+    <t>US-D07
+Vérifier la compatibilité avec les outils de l'établissement (ENT, Pronote...).</t>
+  </si>
+  <si>
+    <t>US-D08
+Envoyer des informations ou recommandations aux enseignants.</t>
+  </si>
+  <si>
+    <t>US-D09
+Comparer les statistiques entre plusieurs années scolaires.</t>
+  </si>
+  <si>
+    <t>US-D10
+Gérer les données d'autres établissements.</t>
+  </si>
+  <si>
+    <t>US-D11
+Former automatiquement les enseignants.</t>
+  </si>
+  <si>
+    <t>US-D12
+Gérer les budgets de plusieurs académies.</t>
   </si>
 </sst>
 </file>
@@ -533,6 +590,30 @@
     <xf numFmtId="0" fontId="8" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -547,9 +628,6 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -558,27 +636,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -890,47 +947,49 @@
     <col min="8" max="8" width="30.140625" customWidth="1"/>
     <col min="9" max="9" width="34.5703125" customWidth="1"/>
     <col min="10" max="10" width="33.28515625" customWidth="1"/>
+    <col min="11" max="11" width="24.7109375" customWidth="1"/>
+    <col min="12" max="13" width="24.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
     </row>
     <row r="2" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
     </row>
     <row r="3" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -955,14 +1014,23 @@
       <c r="G4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="26" t="s">
+      <c r="H4" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="I4" s="26" t="s">
+      <c r="I4" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="J4" s="26" t="s">
+      <c r="J4" s="16" t="s">
         <v>59</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="L4" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="M4" s="16" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
@@ -987,14 +1055,23 @@
       <c r="G5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="27" t="s">
+      <c r="H5" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="I5" s="27" t="s">
+      <c r="I5" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J5" s="27" t="s">
+      <c r="J5" s="17" t="s">
         <v>63</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
@@ -1019,14 +1096,23 @@
       <c r="G6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="I6" s="30" t="s">
+      <c r="I6" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="J6" s="30" t="s">
+      <c r="J6" s="18" t="s">
         <v>66</v>
+      </c>
+      <c r="K6" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="L6" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="M6" s="18" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
@@ -1051,14 +1137,23 @@
       <c r="G7" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="31" t="s">
+      <c r="H7" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="I7" s="31" t="s">
+      <c r="I7" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="J7" s="31" t="s">
+      <c r="J7" s="19" t="s">
         <v>69</v>
+      </c>
+      <c r="K7" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="L7" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="M7" s="19" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
@@ -1083,177 +1178,186 @@
       <c r="G8" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="32" t="s">
+      <c r="H8" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="I8" s="32" t="s">
+      <c r="I8" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="J8" s="32" t="s">
+      <c r="J8" s="20" t="s">
         <v>61</v>
+      </c>
+      <c r="K8" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="L8" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="M8" s="20" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
     </row>
     <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
     </row>
     <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
     </row>
     <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
     </row>
     <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
     </row>
     <row r="15" spans="1:16" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
     </row>
     <row r="17" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
     </row>
     <row r="18" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
     </row>
     <row r="19" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
     </row>
     <row r="20" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
     </row>
     <row r="21" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="16"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
     </row>
     <row r="22" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="15"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="16">

</xml_diff>